<commit_message>
Refactoring of bolts assessment
</commit_message>
<xml_diff>
--- a/src/cassy/additional_data/materials/SS660 (non leak-tight).xlsx
+++ b/src/cassy/additional_data/materials/SS660 (non leak-tight).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d.laghi\Documents\GitHub\StressAssessment\src\kaiser\additional_data\materials\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\laghida\Documents\GitLab\cassy\src\cassy\additional_data\materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8286497-62C9-4260-A064-BF94DC318541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6803A9FB-E7BA-417B-BED6-E4BF66851D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="61590" yWindow="885" windowWidth="21030" windowHeight="13155" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sd_nopeak" sheetId="13" r:id="rId1"/>
@@ -98,9 +98,6 @@
     <t>Sd, irr [Mpa]</t>
   </si>
   <si>
-    <t>stress</t>
-  </si>
-  <si>
     <t>No limit</t>
   </si>
   <si>
@@ -140,6 +137,9 @@
   </si>
   <si>
     <t>K eps [A3.10S.462]</t>
+  </si>
+  <si>
+    <t>strain</t>
   </si>
 </sst>
 </file>
@@ -800,7 +800,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -955,9 +955,6 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="11" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -979,9 +976,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -989,6 +983,33 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="11" fontId="2" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="4" borderId="33" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1031,21 +1052,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="11" fontId="2" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1061,9 +1070,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema di Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1101,7 +1110,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1207,7 +1216,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1349,7 +1358,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1358,33 +1367,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56BE78E7-22BA-45C1-94DB-9B08B5302077}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A2" s="36"/>
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
-    </row>
-    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+    </row>
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="38" t="s">
         <v>9</v>
       </c>
@@ -1422,7 +1431,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A4" s="42">
         <v>20</v>
       </c>
@@ -1460,7 +1469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A5" s="43">
         <v>50</v>
       </c>
@@ -1498,7 +1507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A6" s="43">
         <v>100</v>
       </c>
@@ -1536,7 +1545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A7" s="43">
         <v>150</v>
       </c>
@@ -1574,7 +1583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A8" s="43">
         <v>200</v>
       </c>
@@ -1612,7 +1621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A9" s="43">
         <v>250</v>
       </c>
@@ -1650,7 +1659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A10" s="43">
         <v>300</v>
       </c>
@@ -1688,7 +1697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A11" s="44">
         <v>350</v>
       </c>
@@ -1737,39 +1746,39 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="16.6640625" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="2" width="16.69140625" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B1" s="8"/>
-      <c r="C1" s="72" t="s">
+      <c r="C1" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-    </row>
-    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="80"/>
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
+      <c r="J1" s="80"/>
+      <c r="K1" s="80"/>
+      <c r="L1" s="80"/>
+      <c r="M1" s="80"/>
+      <c r="N1" s="80"/>
+      <c r="O1" s="80"/>
+      <c r="P1" s="80"/>
+    </row>
+    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="76">
+      <c r="B2" s="60">
         <v>1000000</v>
       </c>
       <c r="C2" s="10">
@@ -1815,11 +1824,11 @@
         <v>2500000000</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" s="13">
         <v>20</v>
       </c>
-      <c r="B3" s="78">
+      <c r="B3" s="62">
         <v>1</v>
       </c>
       <c r="C3" s="14">
@@ -1865,11 +1874,11 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="15">
         <v>600</v>
       </c>
-      <c r="B4" s="79">
+      <c r="B4" s="63">
         <v>1</v>
       </c>
       <c r="C4" s="14">
@@ -1926,38 +1935,38 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:P4"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B1" s="8"/>
-      <c r="C1" s="74" t="s">
+      <c r="C1" s="81" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-    </row>
-    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="82"/>
+      <c r="H1" s="82"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="82"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="82"/>
+      <c r="O1" s="82"/>
+      <c r="P1" s="82"/>
+    </row>
+    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="76">
+      <c r="B2" s="60">
         <v>1000000</v>
       </c>
       <c r="C2" s="10">
@@ -2003,11 +2012,11 @@
         <v>2500000000</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" s="13">
         <v>20</v>
       </c>
-      <c r="B3" s="77">
+      <c r="B3" s="61">
         <v>1</v>
       </c>
       <c r="C3" s="16">
@@ -2053,11 +2062,11 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4" s="17">
         <v>600</v>
       </c>
-      <c r="B4" s="77">
+      <c r="B4" s="61">
         <v>1</v>
       </c>
       <c r="C4" s="16">
@@ -2114,13 +2123,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="12.33203125" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="2" width="12.3046875" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -2131,22 +2140,22 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="20">
         <v>20</v>
       </c>
-      <c r="B2" s="61">
+      <c r="B2" s="59">
         <v>2917000000</v>
       </c>
       <c r="C2" s="21">
         <v>0.122</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="22">
         <v>600</v>
       </c>
-      <c r="B3" s="61">
+      <c r="B3" s="59">
         <v>2917000000</v>
       </c>
       <c r="C3" s="21">
@@ -2161,18 +2170,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" customWidth="1"/>
-    <col min="2" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="13.53515625" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="8.84375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A1" s="35" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>0.3</v>
       </c>
@@ -2185,14 +2194,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="6" width="8.88671875" style="2"/>
-    <col min="7" max="7" width="24.109375" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="6" width="8.84375" style="2"/>
+    <col min="7" max="7" width="24.07421875" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2200,7 +2209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" s="24">
         <v>-300</v>
       </c>
@@ -2208,7 +2217,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>20</v>
       </c>
@@ -2216,7 +2225,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>100</v>
       </c>
@@ -2224,7 +2233,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>150</v>
       </c>
@@ -2232,7 +2241,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>200</v>
       </c>
@@ -2240,7 +2249,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>250</v>
       </c>
@@ -2248,7 +2257,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>300</v>
       </c>
@@ -2256,7 +2265,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>350</v>
       </c>
@@ -2264,7 +2273,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>400</v>
       </c>
@@ -2272,7 +2281,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>450</v>
       </c>
@@ -2280,7 +2289,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>500</v>
       </c>
@@ -2288,7 +2297,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>550</v>
       </c>
@@ -2296,7 +2305,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>600</v>
       </c>
@@ -2304,7 +2313,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A15" s="25">
         <v>100000</v>
       </c>
@@ -2320,39 +2329,39 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="16.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="8.84375" style="1"/>
+    <col min="2" max="2" width="16.765625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.84375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="43.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="72" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="43.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="65" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-    </row>
-    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+    </row>
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="64"/>
-    </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+      <c r="B3" s="70" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="71"/>
+    </row>
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -2363,147 +2372,158 @@
         <v>600</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="57">
-        <v>0</v>
-      </c>
-      <c r="B5" s="59">
-        <v>1.0429999999999999</v>
-      </c>
-      <c r="C5" s="51">
-        <v>1.0429999999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="54">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A5" s="56">
+        <v>0</v>
+      </c>
+      <c r="B5" s="64">
+        <v>100000</v>
+      </c>
+      <c r="C5" s="65">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A6" s="66">
+        <v>0</v>
+      </c>
+      <c r="B6" s="67">
+        <v>1.0421</v>
+      </c>
+      <c r="C6" s="68">
+        <v>1.0421</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A7" s="53">
         <v>10</v>
       </c>
-      <c r="B6" s="58">
+      <c r="B7" s="57">
         <v>1.042</v>
       </c>
-      <c r="C6" s="55">
+      <c r="C7" s="54">
         <v>1.042</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="54">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A8" s="53">
         <v>30</v>
       </c>
-      <c r="B7" s="58">
+      <c r="B8" s="57">
         <v>0.78820000000000001</v>
       </c>
-      <c r="C7" s="55">
+      <c r="C8" s="54">
         <v>0.78820000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="54">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A9" s="53">
         <v>100</v>
       </c>
-      <c r="B8" s="58">
+      <c r="B9" s="57">
         <v>0.63719999999999999</v>
       </c>
-      <c r="C8" s="55">
+      <c r="C9" s="54">
         <v>0.63719999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="54">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A10" s="53">
         <v>300</v>
       </c>
-      <c r="B9" s="58">
+      <c r="B10" s="57">
         <v>0.46360000000000001</v>
       </c>
-      <c r="C9" s="55">
+      <c r="C10" s="54">
         <v>0.46360000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="54">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A11" s="53">
         <v>1000</v>
       </c>
-      <c r="B10" s="58">
+      <c r="B11" s="57">
         <v>0.35699999999999998</v>
       </c>
-      <c r="C10" s="55">
+      <c r="C11" s="54">
         <v>0.35699999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="54">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A12" s="53">
         <v>3000</v>
       </c>
-      <c r="B11" s="58">
+      <c r="B12" s="57">
         <v>0.3</v>
       </c>
-      <c r="C11" s="55">
+      <c r="C12" s="54">
         <v>0.3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="56">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A13" s="55">
         <v>10000</v>
       </c>
-      <c r="B12" s="58">
+      <c r="B13" s="57">
         <v>0.255</v>
       </c>
-      <c r="C12" s="55">
+      <c r="C13" s="54">
         <v>0.255</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="56">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A14" s="55">
         <v>30000</v>
       </c>
-      <c r="B13" s="58">
+      <c r="B14" s="57">
         <v>0.222</v>
       </c>
-      <c r="C13" s="55">
+      <c r="C14" s="54">
         <v>0.222</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="56">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A15" s="55">
         <v>100000</v>
       </c>
-      <c r="B14" s="58">
+      <c r="B15" s="57">
         <v>0.1915</v>
       </c>
-      <c r="C14" s="55">
+      <c r="C15" s="54">
         <v>0.1915</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="56">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A16" s="55">
         <v>300000</v>
       </c>
-      <c r="B15" s="58">
+      <c r="B16" s="57">
         <v>0.1678</v>
       </c>
-      <c r="C15" s="55">
+      <c r="C16" s="54">
         <v>0.1678</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="56">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A17" s="55">
         <v>1000000</v>
       </c>
-      <c r="B16" s="58">
+      <c r="B17" s="57">
         <v>0.1452</v>
       </c>
-      <c r="C16" s="55">
+      <c r="C17" s="54">
         <v>0.1452</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="52">
+    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="51">
         <v>1000000</v>
       </c>
-      <c r="B17" s="60">
-        <v>0.14510000000000001</v>
-      </c>
-      <c r="C17" s="53">
-        <v>0.14510000000000001</v>
+      <c r="B18" s="58">
+        <v>0</v>
+      </c>
+      <c r="C18" s="52">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2519,26 +2539,26 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCE4581A-3C59-46E7-A0C7-22A3B97D6358}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="3" max="3" width="10.88671875" customWidth="1"/>
+    <col min="3" max="3" width="10.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="68" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="70"/>
-    </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15.45" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="75" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="76"/>
+      <c r="C1" s="77"/>
+    </row>
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="33"/>
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="67"/>
-    </row>
-    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="74"/>
+    </row>
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="27" t="s">
         <v>9</v>
       </c>
@@ -2549,7 +2569,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="32">
         <v>0</v>
       </c>
@@ -2560,7 +2580,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="28">
         <v>20</v>
       </c>
@@ -2571,7 +2591,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="29">
         <v>50</v>
       </c>
@@ -2582,7 +2602,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="29">
         <v>100</v>
       </c>
@@ -2593,7 +2613,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="29">
         <v>150</v>
       </c>
@@ -2604,7 +2624,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="29">
         <v>200</v>
       </c>
@@ -2615,7 +2635,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="29">
         <v>250</v>
       </c>
@@ -2626,7 +2646,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="29">
         <v>300</v>
       </c>
@@ -2637,7 +2657,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="29">
         <v>350</v>
       </c>
@@ -2648,7 +2668,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="29">
         <v>400</v>
       </c>
@@ -2659,7 +2679,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="29">
         <v>450</v>
       </c>
@@ -2670,7 +2690,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="29">
         <v>500</v>
       </c>
@@ -2681,7 +2701,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" s="29">
         <v>550</v>
       </c>
@@ -2692,7 +2712,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" s="29">
         <v>600</v>
       </c>
@@ -2703,7 +2723,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" s="29">
         <v>650</v>
       </c>
@@ -2714,7 +2734,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A19" s="30">
         <v>651</v>
       </c>
@@ -2739,18 +2759,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B23459BE-600F-465A-9C73-696CD2164805}">
   <dimension ref="A2:C10"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="16384" width="8.84375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="62" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B2" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="62"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C2" s="69"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="35" t="s">
         <v>9</v>
       </c>
@@ -2761,7 +2781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>50</v>
       </c>
@@ -2772,7 +2792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>100</v>
       </c>
@@ -2783,7 +2803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>150</v>
       </c>
@@ -2794,7 +2814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>200</v>
       </c>
@@ -2805,7 +2825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>250</v>
       </c>
@@ -2816,7 +2836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>300</v>
       </c>
@@ -2827,7 +2847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>350</v>
       </c>
@@ -2850,27 +2870,27 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29F8B7B7-B490-4CD3-AB1A-AACEAE39BE05}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="13.3046875" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="8.84375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="62" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B2" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="62"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C2" s="69"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="35" t="s">
         <v>9</v>
       </c>
@@ -2881,7 +2901,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="35">
         <v>20</v>
       </c>
@@ -2892,7 +2912,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="35">
         <v>50</v>
       </c>
@@ -2903,7 +2923,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="35">
         <v>100</v>
       </c>
@@ -2914,7 +2934,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="35">
         <v>150</v>
       </c>
@@ -2925,7 +2945,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="35">
         <v>200</v>
       </c>
@@ -2936,7 +2956,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="35">
         <v>250</v>
       </c>
@@ -2947,7 +2967,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="35">
         <v>300</v>
       </c>
@@ -2958,7 +2978,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="35">
         <v>350</v>
       </c>
@@ -2969,7 +2989,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="35">
         <v>400</v>
       </c>
@@ -2980,7 +3000,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="35">
         <v>450</v>
       </c>
@@ -2991,7 +3011,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="35">
         <v>500</v>
       </c>
@@ -3002,7 +3022,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="35">
         <v>550</v>
       </c>
@@ -3013,7 +3033,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" s="35">
         <v>600</v>
       </c>
@@ -3024,7 +3044,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" s="35">
         <v>650</v>
       </c>
@@ -3047,25 +3067,25 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE986E78-4B6E-4E72-8283-E849FD84C2E5}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="16384" width="8.84375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="62" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="62" t="s">
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B2" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="71"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C2" s="78"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="35" t="s">
         <v>9</v>
       </c>
@@ -3076,7 +3096,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="35">
         <v>20</v>
       </c>
@@ -3087,7 +3107,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="35">
         <v>50</v>
       </c>
@@ -3098,7 +3118,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="35">
         <v>100</v>
       </c>
@@ -3109,7 +3129,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="35">
         <v>150</v>
       </c>
@@ -3120,7 +3140,7 @@
         <v>838</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="35">
         <v>200</v>
       </c>
@@ -3131,7 +3151,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="35">
         <v>250</v>
       </c>
@@ -3142,7 +3162,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="35">
         <v>300</v>
       </c>
@@ -3153,7 +3173,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="35">
         <v>350</v>
       </c>
@@ -3164,7 +3184,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="35">
         <v>400</v>
       </c>
@@ -3175,7 +3195,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="35">
         <v>450</v>
       </c>
@@ -3186,7 +3206,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="35">
         <v>500</v>
       </c>
@@ -3197,7 +3217,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="35">
         <v>550</v>
       </c>
@@ -3208,7 +3228,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" s="35">
         <v>600</v>
       </c>
@@ -3231,33 +3251,33 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46A3757A-8ADF-4E45-B0FD-F8E8977941F9}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A2" s="36"/>
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
-    </row>
-    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+    </row>
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="38" t="s">
         <v>9</v>
       </c>
@@ -3295,308 +3315,308 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A4" s="42">
         <v>20</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L4" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A5" s="43">
         <v>50</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L5" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A6" s="43">
         <v>100</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L6" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A7" s="43">
         <v>150</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L7" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A8" s="43">
         <v>200</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L8" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A9" s="43">
         <v>250</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L9" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A10" s="43">
         <v>300</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L10" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A11" s="44">
         <v>350</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -3610,30 +3630,30 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{039AD92A-97ED-46FD-B28E-A85C9172A402}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A2" s="36"/>
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="69" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
-    </row>
-    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+    </row>
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="38" t="s">
         <v>9</v>
       </c>
@@ -3671,308 +3691,308 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A4" s="42">
         <v>20</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K4" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L4" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A5" s="43">
         <v>50</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K5" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L5" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A6" s="43">
         <v>100</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K6" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L6" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A7" s="43">
         <v>150</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K7" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L7" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A8" s="43">
         <v>200</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K8" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L8" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A9" s="43">
         <v>250</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K9" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L9" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A10" s="43">
         <v>300</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L10" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A11" s="44">
         <v>350</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L11" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -4238,6 +4258,8 @@
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f41f4605-e15c-4135-bd96-d3970596b173"/>
+    <ds:schemaRef ds:uri="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4251,5 +4273,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B71B889C-8F90-4794-ABB2-12F646B3060E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B71B889C-8F90-4794-ABB2-12F646B3060E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
+    <ds:schemaRef ds:uri="f41f4605-e15c-4135-bd96-d3970596b173"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>